<commit_message>
Daily slate 2026-05-21 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-14.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-14.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="E2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G2" t="n">
-        <v>41.2</v>
+        <v>36.4</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E3" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F3" t="n">
         <v>13</v>
       </c>
       <c r="G3" t="n">
-        <v>56.7</v>
+        <v>58.1</v>
       </c>
     </row>
     <row r="4">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>66.7</v>
+        <v>85.7</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="E6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F6" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G6" t="n">
-        <v>41.2</v>
+        <v>45.8</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G7" t="n">
-        <v>37.5</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1099</v>
+        <v>1244</v>
       </c>
       <c r="E8" t="n">
-        <v>216</v>
+        <v>308</v>
       </c>
       <c r="F8" t="n">
-        <v>883</v>
+        <v>936</v>
       </c>
       <c r="G8" t="n">
-        <v>19.7</v>
+        <v>24.8</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>53</v>
+        <v>130</v>
       </c>
       <c r="E9" t="n">
-        <v>20</v>
+        <v>81</v>
       </c>
       <c r="F9" t="n">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="G9" t="n">
-        <v>37.7</v>
+        <v>62.3</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>272</v>
+        <v>388</v>
       </c>
       <c r="E10" t="n">
-        <v>146</v>
+        <v>234</v>
       </c>
       <c r="F10" t="n">
-        <v>126</v>
+        <v>154</v>
       </c>
       <c r="G10" t="n">
-        <v>53.7</v>
+        <v>60.3</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>159</v>
+        <v>244</v>
       </c>
       <c r="E11" t="n">
-        <v>95</v>
+        <v>156</v>
       </c>
       <c r="F11" t="n">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="G11" t="n">
-        <v>59.7</v>
+        <v>63.9</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>66</v>
+        <v>112</v>
       </c>
       <c r="E12" t="n">
-        <v>47</v>
+        <v>83</v>
       </c>
       <c r="F12" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="G12" t="n">
-        <v>71.2</v>
+        <v>74.09999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>22</v>
+        <v>100</v>
       </c>
       <c r="E13" t="n">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="F13" t="n">
-        <v>6</v>
+        <v>49</v>
       </c>
       <c r="G13" t="n">
-        <v>72.7</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="E14" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F14" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G14" t="n">
-        <v>22.4</v>
+        <v>24.3</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="E15" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F15" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G15" t="n">
-        <v>19.1</v>
+        <v>20.8</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G16" t="n">
-        <v>15.8</v>
+        <v>18.2</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>1592</v>
+        <v>1714</v>
       </c>
       <c r="E17" t="n">
-        <v>355</v>
+        <v>390</v>
       </c>
       <c r="F17" t="n">
-        <v>1237</v>
+        <v>1324</v>
       </c>
       <c r="G17" t="n">
-        <v>22.3</v>
+        <v>22.8</v>
       </c>
     </row>
   </sheetData>
@@ -1206,28 +1206,31 @@
         <v>0</v>
       </c>
       <c r="X3" t="n">
-        <v>16.8</v>
+        <v>23</v>
       </c>
       <c r="Y3" t="n">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="Z3" t="n">
-        <v>0</v>
+        <v>33.3</v>
       </c>
       <c r="AA3" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>100</v>
       </c>
       <c r="AC3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AE3" t="n">
         <v>0</v>
       </c>
       <c r="AF3" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="AG3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -1426,58 +1429,58 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>53.7</v>
+        <v>60.3</v>
       </c>
       <c r="C7" t="n">
-        <v>272</v>
+        <v>388</v>
       </c>
       <c r="D7" t="n">
-        <v>59.7</v>
+        <v>63.9</v>
       </c>
       <c r="E7" t="n">
-        <v>159</v>
+        <v>244</v>
       </c>
       <c r="F7" t="n">
-        <v>71.2</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>66</v>
+        <v>112</v>
       </c>
       <c r="H7" t="n">
-        <v>72.7</v>
+        <v>51</v>
       </c>
       <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="K7" t="n">
+        <v>107</v>
+      </c>
+      <c r="L7" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="M7" t="n">
+        <v>101</v>
+      </c>
+      <c r="N7" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="O7" t="n">
         <v>22</v>
       </c>
-      <c r="J7" t="n">
-        <v>22.4</v>
-      </c>
-      <c r="K7" t="n">
-        <v>98</v>
-      </c>
-      <c r="L7" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="M7" t="n">
-        <v>94</v>
-      </c>
-      <c r="N7" t="n">
-        <v>15.8</v>
-      </c>
-      <c r="O7" t="n">
-        <v>19</v>
-      </c>
       <c r="P7" t="n">
-        <v>22.3</v>
+        <v>22.8</v>
       </c>
       <c r="Q7" t="n">
-        <v>1592</v>
+        <v>1714</v>
       </c>
       <c r="R7" t="n">
-        <v>41.2</v>
+        <v>36.4</v>
       </c>
       <c r="S7" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="T7" t="n">
         <v>50</v>
@@ -1486,40 +1489,40 @@
         <v>8</v>
       </c>
       <c r="V7" t="n">
-        <v>41.2</v>
+        <v>45.8</v>
       </c>
       <c r="W7" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="X7" t="n">
-        <v>19.7</v>
+        <v>24.8</v>
       </c>
       <c r="Y7" t="n">
-        <v>1099</v>
+        <v>1244</v>
       </c>
       <c r="Z7" t="n">
-        <v>56.7</v>
+        <v>58.1</v>
       </c>
       <c r="AA7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="AB7" t="n">
-        <v>66.7</v>
+        <v>85.7</v>
       </c>
       <c r="AC7" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AD7" t="n">
-        <v>37.5</v>
+        <v>40</v>
       </c>
       <c r="AE7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AF7" t="n">
-        <v>37.7</v>
+        <v>62.3</v>
       </c>
       <c r="AG7" t="n">
-        <v>53</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>